<commit_message>
Parametreler dosyası eklendi ve Dosyaların açılacağı path değeri dinamik duruma getirildi.
</commit_message>
<xml_diff>
--- a/ExcelSamples/Parametreler.xlsx
+++ b/ExcelSamples/Parametreler.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24465" windowHeight="5640"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -19,14 +20,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>DosyaYeri</t>
   </si>
   <si>
-    <t>D:\</t>
-  </si>
-  <si>
     <t>id</t>
   </si>
   <si>
@@ -40,6 +38,15 @@
   </si>
   <si>
     <t>fileDialog ile dosyalar yüklenirken açılacak yeri gösterir.</t>
+  </si>
+  <si>
+    <t>D:\KorayBey</t>
+  </si>
+  <si>
+    <t>Miktar ve gizlilik verilerinin bulunduğu dosya seçileceği zaman FileDialog için default dizini gösterir.</t>
+  </si>
+  <si>
+    <t>.</t>
   </si>
 </sst>
 </file>
@@ -390,21 +397,22 @@
   <cols>
     <col min="1" max="1" width="6.28515625" customWidth="1"/>
     <col min="2" max="2" width="13.85546875" customWidth="1"/>
-    <col min="4" max="4" width="52.42578125" customWidth="1"/>
+    <col min="3" max="3" width="49" customWidth="1"/>
+    <col min="4" max="4" width="90.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>4</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -415,17 +423,23 @@
         <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
       <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
+      <c r="C3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>

</xml_diff>